<commit_message>
Separate notification routing task from QA gates
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R42cd0e45f6834fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Red2d639e9f274ef4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
         <x:v>任务ID</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
-        <x:v>sqlite_notification_budget_decision_audit</x:v>
+        <x:v>sqlite_notification_budget_routing</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="50" customHeight="1">
@@ -487,33 +487,25 @@
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>失败收口</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>输入数据库、规则或完成版SQL缺失或无效时返回非零状态，删除notify_plan.db和reports目录，保留完成版SQL便于修正</x:v>
+        <x:v>五张源表未变，每个候选只进入发送计划或抑制审计一处，活动余量不为负，三份CSV与数据库派生表一致</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>业务核对</x:v>
       </x:c>
       <x:c r="B18" s="21" t="str">
-        <x:v>五张源表未变，每个候选只进入发送计划或抑制审计一处，活动余量不为负，三份CSV与数据库派生表一致</x:v>
+        <x:v>SQLite版本；源表结构与行；裁决覆盖；本地时间；原因次序；去重窗口；两级配额；唯一索引；报表列序与排序</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>不适合作为评分点的内容</x:v>
       </x:c>
       <x:c r="B19" s="21" t="str">
-        <x:v>SQLite版本；源表结构与行；裁决覆盖；本地时间；原因次序；去重窗口；两级配额；唯一索引；报表列序与排序；重复运行结果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="58" customHeight="1">
-      <x:c r="A20" s="14" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B20" s="21" t="str">
         <x:v>SQL缩进、别名、注释、内部公用表表达式拆分、索引名称、数据库页布局、LF或CRLF差异和不改变业务结果的日志</x:v>
       </x:c>
     </x:row>

</xml_diff>